<commit_message>
Centralize Fall 2026 schedule generation
</commit_message>
<xml_diff>
--- a/data/AD698-Schedule.xlsx
+++ b/data/AD698-Schedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Repositories\AD698-generative-ai-for-BA\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4698A721-042B-4813-B153-1CED8B23E998}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05299E67-D811-45A3-9251-772CA783FE34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-225" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{289CF049-F2D7-49EE-A36E-C623D66A4696}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{289CF049-F2D7-49EE-A36E-C623D66A4696}"/>
   </bookViews>
   <sheets>
     <sheet name="Course Details" sheetId="2" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="282">
   <si>
     <t>Assignment</t>
   </si>
@@ -296,9 +296,6 @@
   </si>
   <si>
     <t>Nakul Padalkar</t>
-  </si>
-  <si>
-    <t>Mon</t>
   </si>
   <si>
     <t>Tue</t>
@@ -1669,10 +1666,10 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="56" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B1" s="60" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C1" s="56" t="s">
         <v>5</v>
@@ -1684,326 +1681,326 @@
         <v>76</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B2" s="60" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D2" s="60" t="s">
+        <v>275</v>
+      </c>
+      <c r="E2" s="60" t="s">
         <v>276</v>
-      </c>
-      <c r="E2" s="60" t="s">
-        <v>277</v>
       </c>
       <c r="F2" s="58"/>
       <c r="G2" s="58"/>
     </row>
     <row r="3" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B3" s="60" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D3" s="60" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E3" s="60" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F3" s="58"/>
       <c r="G3" s="58"/>
     </row>
     <row r="4" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B4" s="60" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D4" s="60" t="s">
+        <v>278</v>
+      </c>
+      <c r="E4" s="60" t="s">
         <v>279</v>
-      </c>
-      <c r="E4" s="60" t="s">
-        <v>280</v>
       </c>
       <c r="F4" s="58"/>
       <c r="G4" s="58"/>
     </row>
     <row r="5" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B5" s="60" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D5" s="60" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E5" s="60" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F5" s="58"/>
       <c r="G5" s="58"/>
     </row>
     <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B6" s="60" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D6" s="60" t="s">
+        <v>215</v>
+      </c>
+      <c r="E6" s="60" t="s">
         <v>216</v>
-      </c>
-      <c r="E6" s="60" t="s">
-        <v>217</v>
       </c>
       <c r="F6" s="58"/>
       <c r="G6" s="58"/>
     </row>
     <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B7" s="60" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D7" s="60" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E7" s="60" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F7" s="58"/>
       <c r="G7" s="58"/>
     </row>
     <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B8" s="60" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D8" s="60" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E8" s="60" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F8" s="58"/>
       <c r="G8" s="58"/>
     </row>
     <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B9" s="60" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D9" s="60" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E9" s="60" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F9" s="58"/>
       <c r="G9" s="58"/>
     </row>
     <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B10" s="60" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D10" s="60" t="s">
+        <v>220</v>
+      </c>
+      <c r="E10" s="60" t="s">
         <v>221</v>
-      </c>
-      <c r="E10" s="60" t="s">
-        <v>222</v>
       </c>
       <c r="F10" s="58"/>
       <c r="G10" s="58"/>
     </row>
     <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B11" s="60" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D11" s="60" t="s">
+        <v>222</v>
+      </c>
+      <c r="E11" s="60" t="s">
         <v>223</v>
-      </c>
-      <c r="E11" s="60" t="s">
-        <v>224</v>
       </c>
       <c r="F11" s="58"/>
       <c r="G11" s="58"/>
     </row>
     <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B12" s="60" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D12" s="60" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E12" s="60" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="F12" s="58"/>
       <c r="G12" s="58"/>
     </row>
     <row r="13" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B13" s="60" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D13" s="60" t="s">
+        <v>225</v>
+      </c>
+      <c r="E13" s="60" t="s">
         <v>226</v>
-      </c>
-      <c r="E13" s="60" t="s">
-        <v>227</v>
       </c>
       <c r="F13" s="58"/>
     </row>
     <row r="14" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B14" s="60" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D14" s="60" t="s">
+        <v>227</v>
+      </c>
+      <c r="E14" s="60" t="s">
         <v>228</v>
-      </c>
-      <c r="E14" s="60" t="s">
-        <v>229</v>
       </c>
       <c r="F14" s="58"/>
     </row>
     <row r="15" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B15" s="60" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D15" s="60" t="s">
+        <v>229</v>
+      </c>
+      <c r="E15" s="60" t="s">
         <v>230</v>
-      </c>
-      <c r="E15" s="60" t="s">
-        <v>231</v>
       </c>
       <c r="F15" s="58"/>
     </row>
     <row r="16" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B16" s="60" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D16" s="60" t="s">
+        <v>231</v>
+      </c>
+      <c r="E16" s="60" t="s">
         <v>232</v>
-      </c>
-      <c r="E16" s="60" t="s">
-        <v>233</v>
       </c>
       <c r="F16" s="58"/>
     </row>
     <row r="17" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B17" s="60" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D17" s="60" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E17" s="60" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F17" s="58"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B18" s="60" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D18" s="60" t="s">
+        <v>237</v>
+      </c>
+      <c r="E18" s="60" t="s">
         <v>238</v>
-      </c>
-      <c r="E18" s="60" t="s">
-        <v>239</v>
       </c>
       <c r="F18" s="58"/>
     </row>
@@ -2052,7 +2049,7 @@
         <v>82</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>83</v>
@@ -2061,24 +2058,24 @@
         <v>84</v>
       </c>
       <c r="E2" s="55" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="54" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>83</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E3" s="55" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
   </sheetData>
@@ -2104,30 +2101,30 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B1" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="C1" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="E1" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="F1" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="G1" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="H1" s="7" t="s">
         <v>91</v>
-      </c>
-      <c r="H1" s="7" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B2" s="9">
         <f>F2</f>
@@ -2138,7 +2135,7 @@
         <v>100</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F2" s="9">
         <v>1</v>
@@ -2153,7 +2150,7 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B3" s="7">
         <v>1</v>
@@ -2162,7 +2159,7 @@
         <v>50</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F3" s="7">
         <v>1</v>
@@ -2177,7 +2174,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B4" s="9">
         <f>F4</f>
@@ -2203,7 +2200,7 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B5" s="9">
         <f>SUM(F6:F9)</f>
@@ -2214,7 +2211,7 @@
         <v>150</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F5" s="9">
         <v>1</v>
@@ -2229,14 +2226,14 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C6" s="9">
         <f>SUM(C2:C5)</f>
         <v>500</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F6" s="9">
         <v>1</v>
@@ -2246,7 +2243,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E7" s="11" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F7" s="9">
         <v>1</v>
@@ -2256,7 +2253,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E8" s="11" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F8" s="9">
         <v>1</v>
@@ -2266,7 +2263,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E9" s="11" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F9" s="9">
         <v>1</v>
@@ -2276,7 +2273,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F10" s="9">
         <v>1</v>
@@ -2291,7 +2288,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E11" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F11" s="9">
         <v>1</v>
@@ -2306,7 +2303,7 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="E12" s="8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F12" s="9"/>
       <c r="G12" s="9"/>
@@ -2335,10 +2332,10 @@
         <v>82</v>
       </c>
       <c r="B1" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="C1" s="13" t="s">
         <v>100</v>
-      </c>
-      <c r="C1" s="13" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -2465,81 +2462,81 @@
   <sheetData>
     <row r="1" spans="1:20" s="15" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="B1" s="16" t="s">
         <v>102</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="C1" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="D1" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="E1" s="15" t="s">
         <v>105</v>
-      </c>
-      <c r="E1" s="15" t="s">
-        <v>106</v>
       </c>
       <c r="F1" s="15" t="s">
         <v>81</v>
       </c>
       <c r="G1" s="17" t="s">
+        <v>106</v>
+      </c>
+      <c r="H1" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="H1" s="18" t="s">
+      <c r="I1" s="18" t="s">
         <v>108</v>
       </c>
-      <c r="I1" s="18" t="s">
+      <c r="J1" s="18" t="s">
         <v>109</v>
       </c>
-      <c r="J1" s="18" t="s">
+      <c r="K1" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="K1" s="18" t="s">
+      <c r="L1" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="L1" s="18" t="s">
+      <c r="M1" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="M1" s="18" t="s">
+      <c r="N1" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="N1" s="18" t="s">
+      <c r="O1" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="O1" s="18" t="s">
+      <c r="P1" s="18" t="s">
         <v>115</v>
       </c>
-      <c r="P1" s="18" t="s">
+      <c r="Q1" s="18" t="s">
         <v>116</v>
       </c>
-      <c r="Q1" s="18" t="s">
+      <c r="R1" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="R1" s="18" t="s">
+      <c r="S1" s="18" t="s">
         <v>118</v>
       </c>
-      <c r="S1" s="18" t="s">
+      <c r="T1" s="19" t="s">
         <v>119</v>
-      </c>
-      <c r="T1" s="19" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
+        <v>120</v>
+      </c>
+      <c r="B2" s="20" t="s">
         <v>121</v>
       </c>
-      <c r="B2" s="20" t="s">
+      <c r="C2" s="20" t="s">
         <v>122</v>
       </c>
-      <c r="C2" s="20" t="s">
+      <c r="D2" s="21" t="s">
         <v>123</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="E2" s="22" t="s">
         <v>124</v>
-      </c>
-      <c r="E2" s="22" t="s">
-        <v>125</v>
       </c>
       <c r="F2" s="23">
         <v>0.60416666666666663</v>
@@ -2598,19 +2595,19 @@
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="20" t="s">
+        <v>125</v>
+      </c>
+      <c r="B3" s="20" t="s">
+        <v>121</v>
+      </c>
+      <c r="C3" s="20" t="s">
+        <v>122</v>
+      </c>
+      <c r="D3" s="21" t="s">
+        <v>123</v>
+      </c>
+      <c r="E3" s="22" t="s">
         <v>126</v>
-      </c>
-      <c r="B3" s="20" t="s">
-        <v>122</v>
-      </c>
-      <c r="C3" s="20" t="s">
-        <v>123</v>
-      </c>
-      <c r="D3" s="21" t="s">
-        <v>124</v>
-      </c>
-      <c r="E3" s="22" t="s">
-        <v>127</v>
       </c>
       <c r="F3" s="25">
         <v>0.79166666666666663</v>
@@ -2695,55 +2692,55 @@
   <sheetData>
     <row r="1" spans="1:17" s="29" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="26" t="s">
+        <v>127</v>
+      </c>
+      <c r="B1" s="27" t="s">
         <v>128</v>
       </c>
-      <c r="B1" s="27" t="s">
+      <c r="C1" s="28" t="s">
+        <v>105</v>
+      </c>
+      <c r="D1" s="18" t="s">
         <v>129</v>
       </c>
-      <c r="C1" s="28" t="s">
-        <v>106</v>
-      </c>
-      <c r="D1" s="18" t="s">
+      <c r="E1" s="18" t="s">
         <v>130</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="F1" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="F1" s="18" t="s">
+      <c r="G1" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="G1" s="18" t="s">
+      <c r="H1" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="H1" s="18" t="s">
+      <c r="I1" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="I1" s="18" t="s">
+      <c r="J1" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="J1" s="18" t="s">
+      <c r="K1" s="18" t="s">
         <v>136</v>
       </c>
-      <c r="K1" s="18" t="s">
+      <c r="L1" s="18" t="s">
         <v>137</v>
       </c>
-      <c r="L1" s="18" t="s">
+      <c r="M1" s="18" t="s">
         <v>138</v>
       </c>
-      <c r="M1" s="18" t="s">
+      <c r="N1" s="18" t="s">
         <v>139</v>
       </c>
-      <c r="N1" s="18" t="s">
+      <c r="O1" s="18" t="s">
         <v>140</v>
       </c>
-      <c r="O1" s="18" t="s">
+      <c r="P1" s="18" t="s">
         <v>141</v>
       </c>
-      <c r="P1" s="18" t="s">
+      <c r="Q1" s="19" t="s">
         <v>142</v>
-      </c>
-      <c r="Q1" s="19" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
@@ -2751,36 +2748,36 @@
         <v>82</v>
       </c>
       <c r="B2" s="31" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C2" s="32" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D2" s="33" t="s">
+        <v>143</v>
+      </c>
+      <c r="E2" s="33" t="s">
         <v>144</v>
       </c>
-      <c r="E2" s="33" t="s">
+      <c r="F2" s="33" t="s">
         <v>145</v>
       </c>
-      <c r="F2" s="33" t="s">
+      <c r="G2" s="33" t="s">
         <v>146</v>
-      </c>
-      <c r="G2" s="33" t="s">
-        <v>147</v>
       </c>
       <c r="H2" s="33"/>
       <c r="I2" s="33" t="s">
+        <v>147</v>
+      </c>
+      <c r="J2" s="33" t="s">
         <v>148</v>
       </c>
-      <c r="J2" s="33" t="s">
+      <c r="K2" s="33" t="s">
         <v>149</v>
-      </c>
-      <c r="K2" s="33" t="s">
-        <v>150</v>
       </c>
       <c r="L2" s="33"/>
       <c r="M2" s="33" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="N2" s="33"/>
       <c r="O2" s="33"/>
@@ -2789,39 +2786,39 @@
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="30" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B3" s="31" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C3" s="32" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D3" s="35" t="s">
+        <v>143</v>
+      </c>
+      <c r="E3" s="35" t="s">
         <v>144</v>
       </c>
-      <c r="E3" s="35" t="s">
+      <c r="F3" s="35" t="s">
         <v>145</v>
       </c>
-      <c r="F3" s="35" t="s">
+      <c r="G3" s="35" t="s">
         <v>146</v>
-      </c>
-      <c r="G3" s="35" t="s">
-        <v>147</v>
       </c>
       <c r="H3" s="35"/>
       <c r="I3" s="35" t="s">
+        <v>147</v>
+      </c>
+      <c r="J3" s="35" t="s">
         <v>148</v>
       </c>
-      <c r="J3" s="35" t="s">
+      <c r="K3" s="35" t="s">
         <v>149</v>
-      </c>
-      <c r="K3" s="35" t="s">
-        <v>150</v>
       </c>
       <c r="L3" s="35"/>
       <c r="M3" s="35" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="N3" s="35"/>
       <c r="O3" s="35"/>
@@ -2830,39 +2827,39 @@
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="30" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B4" s="31" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C4" s="32" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D4" s="35" t="s">
+        <v>143</v>
+      </c>
+      <c r="E4" s="35" t="s">
         <v>144</v>
       </c>
-      <c r="E4" s="35" t="s">
+      <c r="F4" s="35" t="s">
         <v>145</v>
       </c>
-      <c r="F4" s="35" t="s">
+      <c r="G4" s="35" t="s">
         <v>146</v>
-      </c>
-      <c r="G4" s="35" t="s">
-        <v>147</v>
       </c>
       <c r="H4" s="35"/>
       <c r="I4" s="35" t="s">
+        <v>147</v>
+      </c>
+      <c r="J4" s="35" t="s">
         <v>148</v>
       </c>
-      <c r="J4" s="35" t="s">
+      <c r="K4" s="35" t="s">
         <v>149</v>
-      </c>
-      <c r="K4" s="35" t="s">
-        <v>150</v>
       </c>
       <c r="L4" s="35"/>
       <c r="M4" s="35" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="N4" s="35"/>
       <c r="O4" s="35"/>
@@ -2871,10 +2868,10 @@
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="37" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B5" s="38" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C5" s="39"/>
       <c r="D5" s="40"/>
@@ -2897,89 +2894,89 @@
         <v>82</v>
       </c>
       <c r="B6" s="43" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C6" s="44" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D6" s="33"/>
       <c r="E6" s="33"/>
       <c r="G6" s="33" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H6" s="33"/>
       <c r="I6" s="33"/>
       <c r="K6" s="33" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="L6" s="46"/>
       <c r="M6" s="33"/>
       <c r="N6" s="33" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P6" s="47"/>
       <c r="Q6" s="48"/>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="30" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B7" s="31" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C7" s="32" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D7" s="35"/>
       <c r="E7" s="35"/>
       <c r="G7" s="35" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H7" s="35"/>
       <c r="I7" s="35"/>
       <c r="K7" s="35" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="M7" s="35"/>
       <c r="N7" s="35" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P7" s="49"/>
       <c r="Q7" s="50"/>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="30" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B8" s="31" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C8" s="32" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D8" s="35"/>
       <c r="E8" s="35"/>
       <c r="G8" s="35" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H8" s="35"/>
       <c r="I8" s="35"/>
       <c r="K8" s="35" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="M8" s="35"/>
       <c r="N8" s="35" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="P8" s="49"/>
       <c r="Q8" s="50"/>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="37" t="s">
+        <v>153</v>
+      </c>
+      <c r="B9" s="38" t="s">
         <v>154</v>
-      </c>
-      <c r="B9" s="38" t="s">
-        <v>155</v>
       </c>
       <c r="C9" s="39"/>
       <c r="D9" s="40"/>
@@ -3005,112 +3002,112 @@
         <v>6</v>
       </c>
       <c r="C10" s="44" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D10" s="33"/>
       <c r="E10" s="33" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F10" s="33"/>
       <c r="G10" s="33"/>
       <c r="H10" s="33" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I10" s="33"/>
       <c r="J10" s="33"/>
       <c r="K10" s="33" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="L10" s="33"/>
       <c r="M10" s="33"/>
       <c r="N10" s="33" t="s">
+        <v>161</v>
+      </c>
+      <c r="O10" s="33" t="s">
         <v>162</v>
       </c>
-      <c r="O10" s="33" t="s">
-        <v>163</v>
-      </c>
       <c r="P10" s="33" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="Q10" s="34"/>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="30" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B11" s="31" t="s">
         <v>6</v>
       </c>
       <c r="C11" s="32" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D11" s="35"/>
       <c r="E11" s="35" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F11" s="35"/>
       <c r="G11" s="35"/>
       <c r="H11" s="35" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I11" s="35"/>
       <c r="J11" s="35"/>
       <c r="K11" s="35" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="L11" s="35"/>
       <c r="M11" s="35"/>
       <c r="N11" s="35" t="s">
+        <v>161</v>
+      </c>
+      <c r="O11" s="35" t="s">
         <v>162</v>
       </c>
-      <c r="O11" s="35" t="s">
-        <v>163</v>
-      </c>
       <c r="P11" s="35" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="Q11" s="36"/>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="30" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B12" s="31" t="s">
         <v>6</v>
       </c>
       <c r="C12" s="32" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D12" s="35"/>
       <c r="E12" s="35" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F12" s="35"/>
       <c r="G12" s="35"/>
       <c r="H12" s="35" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I12" s="35"/>
       <c r="J12" s="35"/>
       <c r="K12" s="35" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="L12" s="35"/>
       <c r="M12" s="35"/>
       <c r="N12" s="35" t="s">
+        <v>161</v>
+      </c>
+      <c r="O12" s="35" t="s">
         <v>162</v>
       </c>
-      <c r="O12" s="35" t="s">
-        <v>163</v>
-      </c>
       <c r="P12" s="35" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="Q12" s="36"/>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="37" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B13" s="38" t="s">
         <v>6</v>
@@ -3136,10 +3133,10 @@
         <v>82</v>
       </c>
       <c r="B14" s="43" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C14" s="44" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D14" s="33"/>
       <c r="E14" s="33"/>
@@ -3151,7 +3148,7 @@
       <c r="K14" s="46"/>
       <c r="L14" s="33"/>
       <c r="M14" s="33" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="N14" s="33"/>
       <c r="O14" s="33"/>
@@ -3160,13 +3157,13 @@
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="30" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B15" s="31" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C15" s="32" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D15" s="35"/>
       <c r="E15" s="35"/>
@@ -3177,7 +3174,7 @@
       <c r="J15" s="35"/>
       <c r="L15" s="35"/>
       <c r="M15" s="35" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="N15" s="35"/>
       <c r="O15" s="35"/>
@@ -3186,13 +3183,13 @@
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="30" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B16" s="31" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C16" s="32" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D16" s="35"/>
       <c r="E16" s="35"/>
@@ -3203,7 +3200,7 @@
       <c r="J16" s="35"/>
       <c r="L16" s="35"/>
       <c r="M16" s="35" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="N16" s="35"/>
       <c r="O16" s="35"/>
@@ -3212,10 +3209,10 @@
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="37" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B17" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C17" s="39"/>
       <c r="D17" s="40"/>
@@ -3228,7 +3225,7 @@
       <c r="K17" s="40"/>
       <c r="L17" s="40"/>
       <c r="M17" s="40" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="N17" s="40"/>
       <c r="O17" s="40"/>
@@ -3240,10 +3237,10 @@
         <v>82</v>
       </c>
       <c r="B18" s="31" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C18" s="32" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D18" s="35"/>
       <c r="F18" s="35"/>
@@ -3254,7 +3251,7 @@
       <c r="K18" s="35"/>
       <c r="L18" s="35"/>
       <c r="M18" s="35" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="N18" s="35"/>
       <c r="O18" s="35"/>
@@ -3263,13 +3260,13 @@
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="30" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B19" s="31" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C19" s="32" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D19" s="35"/>
       <c r="F19" s="35"/>
@@ -3280,7 +3277,7 @@
       <c r="K19" s="35"/>
       <c r="L19" s="35"/>
       <c r="M19" s="35" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="N19" s="35"/>
       <c r="O19" s="35"/>
@@ -3289,13 +3286,13 @@
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="30" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B20" s="31" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C20" s="32" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D20" s="35"/>
       <c r="F20" s="35"/>
@@ -3306,7 +3303,7 @@
       <c r="K20" s="35"/>
       <c r="L20" s="35"/>
       <c r="M20" s="35" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="N20" s="35"/>
       <c r="O20" s="35"/>
@@ -3315,10 +3312,10 @@
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="37" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B21" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C21" s="39"/>
       <c r="D21" s="40"/>
@@ -3331,7 +3328,7 @@
       <c r="K21" s="40"/>
       <c r="L21" s="40"/>
       <c r="M21" s="40" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="N21" s="40"/>
       <c r="O21" s="40"/>
@@ -3359,7 +3356,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="56" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B1" s="56" t="s">
         <v>5</v>
@@ -3371,10 +3368,10 @@
         <v>76</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>169</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -3674,97 +3671,97 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
   </sheetData>
@@ -3789,10 +3786,10 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="56" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B1" s="59" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C1" s="56" t="s">
         <v>5</v>
@@ -3804,364 +3801,364 @@
         <v>76</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B2" s="59" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D2" s="57" t="s">
+        <v>270</v>
+      </c>
+      <c r="E2" s="57" t="s">
         <v>271</v>
-      </c>
-      <c r="E2" s="57" t="s">
-        <v>272</v>
       </c>
       <c r="F2" s="58"/>
       <c r="G2" s="58"/>
     </row>
     <row r="3" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B3" s="59" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D3" s="57" t="s">
+        <v>268</v>
+      </c>
+      <c r="E3" s="57" t="s">
         <v>269</v>
-      </c>
-      <c r="E3" s="57" t="s">
-        <v>270</v>
       </c>
       <c r="F3" s="58"/>
       <c r="G3" s="58"/>
     </row>
     <row r="4" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B4" s="59" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C4" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>273</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="E4" s="60" t="s">
         <v>274</v>
-      </c>
-      <c r="E4" s="60" t="s">
-        <v>275</v>
       </c>
       <c r="F4" s="58"/>
       <c r="G4" s="58"/>
     </row>
     <row r="5" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B5" s="59" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D5" s="59" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E5" s="59" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F5" s="58"/>
       <c r="G5" s="58"/>
     </row>
     <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B6" s="59" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D6" s="59" t="s">
+        <v>215</v>
+      </c>
+      <c r="E6" s="59" t="s">
         <v>216</v>
-      </c>
-      <c r="E6" s="59" t="s">
-        <v>217</v>
       </c>
       <c r="F6" s="58"/>
       <c r="G6" s="58"/>
     </row>
     <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B7" s="59" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D7" s="59" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E7" s="59" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F7" s="58"/>
       <c r="G7" s="58"/>
     </row>
     <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B8" s="59" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D8" s="59" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E8" s="59" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F8" s="58"/>
       <c r="G8" s="58"/>
     </row>
     <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B9" s="59" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D9" s="59" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E9" s="59" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F9" s="58"/>
       <c r="G9" s="58"/>
     </row>
     <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B10" s="59" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D10" s="59" t="s">
+        <v>220</v>
+      </c>
+      <c r="E10" s="59" t="s">
         <v>221</v>
-      </c>
-      <c r="E10" s="59" t="s">
-        <v>222</v>
       </c>
       <c r="F10" s="58"/>
       <c r="G10" s="58"/>
     </row>
     <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B11" s="59" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D11" s="59" t="s">
+        <v>222</v>
+      </c>
+      <c r="E11" s="59" t="s">
         <v>223</v>
-      </c>
-      <c r="E11" s="59" t="s">
-        <v>224</v>
       </c>
       <c r="F11" s="58"/>
       <c r="G11" s="58"/>
     </row>
     <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B12" s="59" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D12" s="59" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E12" s="59" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="F12" s="58"/>
       <c r="G12" s="58"/>
     </row>
     <row r="13" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B13" s="59" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D13" s="59" t="s">
+        <v>225</v>
+      </c>
+      <c r="E13" s="59" t="s">
         <v>226</v>
-      </c>
-      <c r="E13" s="59" t="s">
-        <v>227</v>
       </c>
       <c r="F13" s="58"/>
       <c r="G13" s="58"/>
     </row>
     <row r="14" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B14" s="59" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D14" s="59" t="s">
+        <v>227</v>
+      </c>
+      <c r="E14" s="59" t="s">
         <v>228</v>
-      </c>
-      <c r="E14" s="59" t="s">
-        <v>229</v>
       </c>
       <c r="F14" s="58"/>
       <c r="G14" s="58"/>
     </row>
     <row r="15" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B15" s="59" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D15" s="59" t="s">
+        <v>229</v>
+      </c>
+      <c r="E15" s="59" t="s">
         <v>230</v>
-      </c>
-      <c r="E15" s="59" t="s">
-        <v>231</v>
       </c>
       <c r="F15" s="58"/>
     </row>
     <row r="16" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B16" s="59" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D16" s="59" t="s">
+        <v>231</v>
+      </c>
+      <c r="E16" s="59" t="s">
         <v>232</v>
-      </c>
-      <c r="E16" s="59" t="s">
-        <v>233</v>
       </c>
       <c r="F16" s="58"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B17" s="59" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D17" s="59" t="s">
+        <v>233</v>
+      </c>
+      <c r="E17" s="59" t="s">
         <v>234</v>
-      </c>
-      <c r="E17" s="59" t="s">
-        <v>235</v>
       </c>
       <c r="F17" s="58"/>
     </row>
     <row r="18" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B18" s="59" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D18" s="59" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E18" s="59" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F18" s="58"/>
     </row>
     <row r="19" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B19" s="59" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D19" s="59" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E19" s="59" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F19" s="58"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B20" s="59" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D20" s="59" t="s">
+        <v>237</v>
+      </c>
+      <c r="E20" s="59" t="s">
         <v>238</v>
-      </c>
-      <c r="E20" s="59" t="s">
-        <v>239</v>
       </c>
       <c r="F20" s="58"/>
     </row>

</xml_diff>

<commit_message>
fix(schedule): preserve Fall dates and deliverables
</commit_message>
<xml_diff>
--- a/data/AD698-Schedule.xlsx
+++ b/data/AD698-Schedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Repositories\AD698-generative-ai-for-BA\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05299E67-D811-45A3-9251-772CA783FE34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{650E386C-DBBF-4DF3-A076-456BB8BBD2D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{289CF049-F2D7-49EE-A36E-C623D66A4696}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="8" xr2:uid="{289CF049-F2D7-49EE-A36E-C623D66A4696}"/>
   </bookViews>
   <sheets>
     <sheet name="Course Details" sheetId="2" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="281">
   <si>
     <t>Assignment</t>
   </si>
@@ -677,9 +677,6 @@
   </si>
   <si>
     <t>M8</t>
-  </si>
-  <si>
-    <t>O</t>
   </si>
   <si>
     <t>Group Paper Presentation (Once per Group)*</t>
@@ -1669,7 +1666,7 @@
         <v>167</v>
       </c>
       <c r="B1" s="60" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C1" s="56" t="s">
         <v>5</v>
@@ -1692,16 +1689,16 @@
         <v>202</v>
       </c>
       <c r="B2" s="60" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>172</v>
       </c>
       <c r="D2" s="60" t="s">
+        <v>274</v>
+      </c>
+      <c r="E2" s="60" t="s">
         <v>275</v>
-      </c>
-      <c r="E2" s="60" t="s">
-        <v>276</v>
       </c>
       <c r="F2" s="58"/>
       <c r="G2" s="58"/>
@@ -1711,16 +1708,16 @@
         <v>202</v>
       </c>
       <c r="B3" s="60" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>173</v>
       </c>
       <c r="D3" s="60" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E3" s="60" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F3" s="58"/>
       <c r="G3" s="58"/>
@@ -1730,16 +1727,16 @@
         <v>202</v>
       </c>
       <c r="B4" s="60" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D4" s="60" t="s">
+        <v>277</v>
+      </c>
+      <c r="E4" s="60" t="s">
         <v>278</v>
-      </c>
-      <c r="E4" s="60" t="s">
-        <v>279</v>
       </c>
       <c r="F4" s="58"/>
       <c r="G4" s="58"/>
@@ -1749,16 +1746,16 @@
         <v>203</v>
       </c>
       <c r="B5" s="60" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>174</v>
       </c>
       <c r="D5" s="60" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="E5" s="60" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F5" s="58"/>
       <c r="G5" s="58"/>
@@ -1768,16 +1765,16 @@
         <v>203</v>
       </c>
       <c r="B6" s="60" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>175</v>
       </c>
       <c r="D6" s="60" t="s">
+        <v>214</v>
+      </c>
+      <c r="E6" s="60" t="s">
         <v>215</v>
-      </c>
-      <c r="E6" s="60" t="s">
-        <v>216</v>
       </c>
       <c r="F6" s="58"/>
       <c r="G6" s="58"/>
@@ -1787,7 +1784,7 @@
         <v>204</v>
       </c>
       <c r="B7" s="60" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>176</v>
@@ -1796,7 +1793,7 @@
         <v>196</v>
       </c>
       <c r="E7" s="60" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="F7" s="58"/>
       <c r="G7" s="58"/>
@@ -1806,7 +1803,7 @@
         <v>204</v>
       </c>
       <c r="B8" s="60" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>177</v>
@@ -1815,7 +1812,7 @@
         <v>197</v>
       </c>
       <c r="E8" s="60" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F8" s="58"/>
       <c r="G8" s="58"/>
@@ -1825,7 +1822,7 @@
         <v>205</v>
       </c>
       <c r="B9" s="60" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>178</v>
@@ -1834,7 +1831,7 @@
         <v>198</v>
       </c>
       <c r="E9" s="60" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F9" s="58"/>
       <c r="G9" s="58"/>
@@ -1844,16 +1841,16 @@
         <v>205</v>
       </c>
       <c r="B10" s="60" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>179</v>
       </c>
       <c r="D10" s="60" t="s">
+        <v>219</v>
+      </c>
+      <c r="E10" s="60" t="s">
         <v>220</v>
-      </c>
-      <c r="E10" s="60" t="s">
-        <v>221</v>
       </c>
       <c r="F10" s="58"/>
       <c r="G10" s="58"/>
@@ -1863,16 +1860,16 @@
         <v>206</v>
       </c>
       <c r="B11" s="60" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>180</v>
       </c>
       <c r="D11" s="60" t="s">
+        <v>221</v>
+      </c>
+      <c r="E11" s="60" t="s">
         <v>222</v>
-      </c>
-      <c r="E11" s="60" t="s">
-        <v>223</v>
       </c>
       <c r="F11" s="58"/>
       <c r="G11" s="58"/>
@@ -1882,7 +1879,7 @@
         <v>206</v>
       </c>
       <c r="B12" s="60" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>181</v>
@@ -1891,7 +1888,7 @@
         <v>199</v>
       </c>
       <c r="E12" s="60" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="F12" s="58"/>
       <c r="G12" s="58"/>
@@ -1901,16 +1898,16 @@
         <v>207</v>
       </c>
       <c r="B13" s="60" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>182</v>
       </c>
       <c r="D13" s="60" t="s">
+        <v>224</v>
+      </c>
+      <c r="E13" s="60" t="s">
         <v>225</v>
-      </c>
-      <c r="E13" s="60" t="s">
-        <v>226</v>
       </c>
       <c r="F13" s="58"/>
     </row>
@@ -1919,16 +1916,16 @@
         <v>207</v>
       </c>
       <c r="B14" s="60" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>183</v>
       </c>
       <c r="D14" s="60" t="s">
+        <v>226</v>
+      </c>
+      <c r="E14" s="60" t="s">
         <v>227</v>
-      </c>
-      <c r="E14" s="60" t="s">
-        <v>228</v>
       </c>
       <c r="F14" s="58"/>
     </row>
@@ -1937,16 +1934,16 @@
         <v>208</v>
       </c>
       <c r="B15" s="60" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>184</v>
       </c>
       <c r="D15" s="60" t="s">
+        <v>228</v>
+      </c>
+      <c r="E15" s="60" t="s">
         <v>229</v>
-      </c>
-      <c r="E15" s="60" t="s">
-        <v>230</v>
       </c>
       <c r="F15" s="58"/>
     </row>
@@ -1955,16 +1952,16 @@
         <v>208</v>
       </c>
       <c r="B16" s="60" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>185</v>
       </c>
       <c r="D16" s="60" t="s">
+        <v>230</v>
+      </c>
+      <c r="E16" s="60" t="s">
         <v>231</v>
-      </c>
-      <c r="E16" s="60" t="s">
-        <v>232</v>
       </c>
       <c r="F16" s="58"/>
     </row>
@@ -1973,7 +1970,7 @@
         <v>209</v>
       </c>
       <c r="B17" s="60" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>186</v>
@@ -1982,7 +1979,7 @@
         <v>201</v>
       </c>
       <c r="E17" s="60" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F17" s="58"/>
     </row>
@@ -1991,16 +1988,16 @@
         <v>209</v>
       </c>
       <c r="B18" s="60" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>187</v>
       </c>
       <c r="D18" s="60" t="s">
+        <v>236</v>
+      </c>
+      <c r="E18" s="60" t="s">
         <v>237</v>
-      </c>
-      <c r="E18" s="60" t="s">
-        <v>238</v>
       </c>
       <c r="F18" s="58"/>
     </row>
@@ -2016,7 +2013,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF015F21-B674-4B2F-B456-A6FAF27E0BC1}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" style="6" bestFit="1" customWidth="1"/>
@@ -2058,23 +2055,6 @@
         <v>84</v>
       </c>
       <c r="E2" s="55" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="54" t="s">
-        <v>211</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="E3" s="55" t="s">
         <v>190</v>
       </c>
     </row>
@@ -2159,7 +2139,7 @@
         <v>50</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F3" s="7">
         <v>1</v>
@@ -3671,97 +3651,97 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
   </sheetData>
@@ -3789,7 +3769,7 @@
         <v>167</v>
       </c>
       <c r="B1" s="59" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C1" s="56" t="s">
         <v>5</v>
@@ -3812,16 +3792,16 @@
         <v>202</v>
       </c>
       <c r="B2" s="59" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>172</v>
       </c>
       <c r="D2" s="57" t="s">
+        <v>269</v>
+      </c>
+      <c r="E2" s="57" t="s">
         <v>270</v>
-      </c>
-      <c r="E2" s="57" t="s">
-        <v>271</v>
       </c>
       <c r="F2" s="58"/>
       <c r="G2" s="58"/>
@@ -3831,16 +3811,16 @@
         <v>202</v>
       </c>
       <c r="B3" s="59" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>173</v>
       </c>
       <c r="D3" s="57" t="s">
+        <v>267</v>
+      </c>
+      <c r="E3" s="57" t="s">
         <v>268</v>
-      </c>
-      <c r="E3" s="57" t="s">
-        <v>269</v>
       </c>
       <c r="F3" s="58"/>
       <c r="G3" s="58"/>
@@ -3850,16 +3830,16 @@
         <v>202</v>
       </c>
       <c r="B4" s="59" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C4" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>272</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="E4" s="60" t="s">
         <v>273</v>
-      </c>
-      <c r="E4" s="60" t="s">
-        <v>274</v>
       </c>
       <c r="F4" s="58"/>
       <c r="G4" s="58"/>
@@ -3869,16 +3849,16 @@
         <v>203</v>
       </c>
       <c r="B5" s="59" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>174</v>
       </c>
       <c r="D5" s="59" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="E5" s="59" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F5" s="58"/>
       <c r="G5" s="58"/>
@@ -3888,16 +3868,16 @@
         <v>203</v>
       </c>
       <c r="B6" s="59" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>175</v>
       </c>
       <c r="D6" s="59" t="s">
+        <v>214</v>
+      </c>
+      <c r="E6" s="59" t="s">
         <v>215</v>
-      </c>
-      <c r="E6" s="59" t="s">
-        <v>216</v>
       </c>
       <c r="F6" s="58"/>
       <c r="G6" s="58"/>
@@ -3907,7 +3887,7 @@
         <v>204</v>
       </c>
       <c r="B7" s="59" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>176</v>
@@ -3916,7 +3896,7 @@
         <v>196</v>
       </c>
       <c r="E7" s="59" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="F7" s="58"/>
       <c r="G7" s="58"/>
@@ -3926,7 +3906,7 @@
         <v>204</v>
       </c>
       <c r="B8" s="59" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>177</v>
@@ -3935,7 +3915,7 @@
         <v>197</v>
       </c>
       <c r="E8" s="59" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F8" s="58"/>
       <c r="G8" s="58"/>
@@ -3945,7 +3925,7 @@
         <v>205</v>
       </c>
       <c r="B9" s="59" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>178</v>
@@ -3954,7 +3934,7 @@
         <v>198</v>
       </c>
       <c r="E9" s="59" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F9" s="58"/>
       <c r="G9" s="58"/>
@@ -3964,16 +3944,16 @@
         <v>205</v>
       </c>
       <c r="B10" s="59" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>179</v>
       </c>
       <c r="D10" s="59" t="s">
+        <v>219</v>
+      </c>
+      <c r="E10" s="59" t="s">
         <v>220</v>
-      </c>
-      <c r="E10" s="59" t="s">
-        <v>221</v>
       </c>
       <c r="F10" s="58"/>
       <c r="G10" s="58"/>
@@ -3983,16 +3963,16 @@
         <v>206</v>
       </c>
       <c r="B11" s="59" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>180</v>
       </c>
       <c r="D11" s="59" t="s">
+        <v>221</v>
+      </c>
+      <c r="E11" s="59" t="s">
         <v>222</v>
-      </c>
-      <c r="E11" s="59" t="s">
-        <v>223</v>
       </c>
       <c r="F11" s="58"/>
       <c r="G11" s="58"/>
@@ -4002,7 +3982,7 @@
         <v>206</v>
       </c>
       <c r="B12" s="59" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>181</v>
@@ -4011,7 +3991,7 @@
         <v>199</v>
       </c>
       <c r="E12" s="59" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="F12" s="58"/>
       <c r="G12" s="58"/>
@@ -4021,16 +4001,16 @@
         <v>207</v>
       </c>
       <c r="B13" s="59" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>182</v>
       </c>
       <c r="D13" s="59" t="s">
+        <v>224</v>
+      </c>
+      <c r="E13" s="59" t="s">
         <v>225</v>
-      </c>
-      <c r="E13" s="59" t="s">
-        <v>226</v>
       </c>
       <c r="F13" s="58"/>
       <c r="G13" s="58"/>
@@ -4040,16 +4020,16 @@
         <v>207</v>
       </c>
       <c r="B14" s="59" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>183</v>
       </c>
       <c r="D14" s="59" t="s">
+        <v>226</v>
+      </c>
+      <c r="E14" s="59" t="s">
         <v>227</v>
-      </c>
-      <c r="E14" s="59" t="s">
-        <v>228</v>
       </c>
       <c r="F14" s="58"/>
       <c r="G14" s="58"/>
@@ -4059,16 +4039,16 @@
         <v>208</v>
       </c>
       <c r="B15" s="59" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>184</v>
       </c>
       <c r="D15" s="59" t="s">
+        <v>228</v>
+      </c>
+      <c r="E15" s="59" t="s">
         <v>229</v>
-      </c>
-      <c r="E15" s="59" t="s">
-        <v>230</v>
       </c>
       <c r="F15" s="58"/>
     </row>
@@ -4077,16 +4057,16 @@
         <v>208</v>
       </c>
       <c r="B16" s="59" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>185</v>
       </c>
       <c r="D16" s="59" t="s">
+        <v>230</v>
+      </c>
+      <c r="E16" s="59" t="s">
         <v>231</v>
-      </c>
-      <c r="E16" s="59" t="s">
-        <v>232</v>
       </c>
       <c r="F16" s="58"/>
     </row>
@@ -4095,16 +4075,16 @@
         <v>209</v>
       </c>
       <c r="B17" s="59" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>186</v>
       </c>
       <c r="D17" s="59" t="s">
+        <v>232</v>
+      </c>
+      <c r="E17" s="59" t="s">
         <v>233</v>
-      </c>
-      <c r="E17" s="59" t="s">
-        <v>234</v>
       </c>
       <c r="F17" s="58"/>
     </row>
@@ -4113,7 +4093,7 @@
         <v>209</v>
       </c>
       <c r="B18" s="59" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>187</v>
@@ -4122,7 +4102,7 @@
         <v>200</v>
       </c>
       <c r="E18" s="59" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F18" s="58"/>
     </row>
@@ -4131,7 +4111,7 @@
         <v>210</v>
       </c>
       <c r="B19" s="59" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>188</v>
@@ -4140,7 +4120,7 @@
         <v>201</v>
       </c>
       <c r="E19" s="59" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F19" s="58"/>
     </row>
@@ -4149,16 +4129,16 @@
         <v>210</v>
       </c>
       <c r="B20" s="59" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>189</v>
       </c>
       <c r="D20" s="59" t="s">
+        <v>236</v>
+      </c>
+      <c r="E20" s="59" t="s">
         <v>237</v>
-      </c>
-      <c r="E20" s="59" t="s">
-        <v>238</v>
       </c>
       <c r="F20" s="58"/>
     </row>

</xml_diff>